<commit_message>
manipulate excel files to resolve ambiguity
</commit_message>
<xml_diff>
--- a/frontend/public/weekly_contest_2_leaderboard_v2.xlsx
+++ b/frontend/public/weekly_contest_2_leaderboard_v2.xlsx
@@ -1,12 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Anisha Bhat\Documents\Test\Hackerearth_official\frontend\public\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{809C8169-44B2-4D8B-97C8-6F9976C019D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -25,9 +34,6 @@
     <t>Time Taken</t>
   </si>
   <si>
-    <t>Sandeep pai kulyadi</t>
-  </si>
-  <si>
     <t>Ashwitha</t>
   </si>
   <si>
@@ -134,36 +140,38 @@
   </si>
   <si>
     <t>NNM23CB064 SUSHANTH M ALVA</t>
+  </si>
+  <si>
+    <t>Sandeep pai</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="hh:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="d/m"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="d/m"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
     </font>
@@ -173,54 +181,52 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="9">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
+    <xf numFmtId="21" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -410,23 +416,26 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:S38"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="34.75"/>
-    <col customWidth="1" min="2" max="2" width="17.0"/>
-    <col customWidth="1" min="3" max="3" width="16.75"/>
-    <col customWidth="1" min="4" max="4" width="16.0"/>
+    <col min="1" max="1" width="34.77734375" customWidth="1"/>
+    <col min="2" max="2" width="17" customWidth="1"/>
+    <col min="3" max="3" width="16.77734375" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -455,18 +464,18 @@
       <c r="R1" s="1"/>
       <c r="S1" s="1"/>
     </row>
-    <row r="2">
+    <row r="2" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="B2" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="C2" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D2" s="4">
-        <v>0.017638888888888888</v>
+        <v>1.7638888888888888E-2</v>
       </c>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
@@ -479,23 +488,23 @@
       <c r="M2" s="2"/>
       <c r="N2" s="2"/>
       <c r="O2" s="2"/>
-      <c r="P2" s="7"/>
-      <c r="Q2" s="7"/>
-      <c r="R2" s="7"/>
+      <c r="P2" s="2"/>
+      <c r="Q2" s="2"/>
+      <c r="R2" s="2"/>
       <c r="S2" s="2"/>
     </row>
-    <row r="3">
+    <row r="3" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B3" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="C3" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D3" s="4">
-        <v>0.02017361111111111</v>
+        <v>2.0173611111111111E-2</v>
       </c>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
@@ -508,23 +517,23 @@
       <c r="M3" s="2"/>
       <c r="N3" s="2"/>
       <c r="O3" s="2"/>
-      <c r="P3" s="7"/>
-      <c r="Q3" s="7"/>
-      <c r="R3" s="7"/>
+      <c r="P3" s="2"/>
+      <c r="Q3" s="2"/>
+      <c r="R3" s="2"/>
       <c r="S3" s="2"/>
     </row>
-    <row r="4">
+    <row r="4" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B4" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="C4" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D4" s="4">
-        <v>0.020300925925925927</v>
+        <v>2.0300925925925927E-2</v>
       </c>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
@@ -537,23 +546,23 @@
       <c r="M4" s="2"/>
       <c r="N4" s="2"/>
       <c r="O4" s="2"/>
-      <c r="P4" s="7"/>
-      <c r="Q4" s="7"/>
-      <c r="R4" s="7"/>
+      <c r="P4" s="2"/>
+      <c r="Q4" s="2"/>
+      <c r="R4" s="2"/>
       <c r="S4" s="2"/>
     </row>
-    <row r="5">
+    <row r="5" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B5" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="C5" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D5" s="4">
-        <v>0.02392361111111111</v>
+        <v>2.3923611111111111E-2</v>
       </c>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
@@ -566,23 +575,23 @@
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
-      <c r="P5" s="7"/>
-      <c r="Q5" s="7"/>
-      <c r="R5" s="7"/>
+      <c r="P5" s="2"/>
+      <c r="Q5" s="2"/>
+      <c r="R5" s="2"/>
       <c r="S5" s="2"/>
     </row>
-    <row r="6">
+    <row r="6" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B6" s="3">
-        <v>490.0</v>
+        <v>490</v>
       </c>
       <c r="C6" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D6" s="4">
-        <v>0.04607638888888889</v>
+        <v>4.6076388888888889E-2</v>
       </c>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
@@ -595,23 +604,23 @@
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
-      <c r="P6" s="7"/>
-      <c r="Q6" s="7"/>
-      <c r="R6" s="7"/>
+      <c r="P6" s="2"/>
+      <c r="Q6" s="2"/>
+      <c r="R6" s="2"/>
       <c r="S6" s="2"/>
     </row>
-    <row r="7">
+    <row r="7" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B7" s="3">
-        <v>480.0</v>
+        <v>480</v>
       </c>
       <c r="C7" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D7" s="4">
-        <v>0.03152777777777778</v>
+        <v>3.152777777777778E-2</v>
       </c>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
@@ -624,23 +633,23 @@
       <c r="M7" s="2"/>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
-      <c r="P7" s="7"/>
-      <c r="Q7" s="7"/>
-      <c r="R7" s="7"/>
+      <c r="P7" s="2"/>
+      <c r="Q7" s="2"/>
+      <c r="R7" s="2"/>
       <c r="S7" s="2"/>
     </row>
-    <row r="8">
+    <row r="8" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B8" s="3">
-        <v>420.0</v>
+        <v>420</v>
       </c>
       <c r="C8" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D8" s="4">
-        <v>0.06184027777777778</v>
+        <v>6.1840277777777779E-2</v>
       </c>
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
@@ -653,23 +662,23 @@
       <c r="M8" s="2"/>
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
-      <c r="P8" s="7"/>
-      <c r="Q8" s="7"/>
-      <c r="R8" s="7"/>
+      <c r="P8" s="2"/>
+      <c r="Q8" s="2"/>
+      <c r="R8" s="2"/>
       <c r="S8" s="2"/>
     </row>
-    <row r="9">
+    <row r="9" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B9" s="3">
-        <v>410.0</v>
+        <v>410</v>
       </c>
       <c r="C9" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D9" s="4">
-        <v>0.04434027777777778</v>
+        <v>4.4340277777777777E-2</v>
       </c>
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
@@ -682,23 +691,23 @@
       <c r="M9" s="2"/>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
-      <c r="P9" s="7"/>
-      <c r="Q9" s="7"/>
-      <c r="R9" s="7"/>
+      <c r="P9" s="2"/>
+      <c r="Q9" s="2"/>
+      <c r="R9" s="2"/>
       <c r="S9" s="2"/>
     </row>
-    <row r="10">
+    <row r="10" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B10" s="3">
-        <v>400.0</v>
+        <v>400</v>
       </c>
       <c r="C10" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D10" s="4">
-        <v>0.01810185185185185</v>
+        <v>1.8101851851851852E-2</v>
       </c>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
@@ -711,23 +720,23 @@
       <c r="M10" s="2"/>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
-      <c r="P10" s="7"/>
-      <c r="Q10" s="7"/>
-      <c r="R10" s="7"/>
+      <c r="P10" s="2"/>
+      <c r="Q10" s="2"/>
+      <c r="R10" s="2"/>
       <c r="S10" s="2"/>
     </row>
-    <row r="11">
+    <row r="11" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B11" s="3">
-        <v>400.0</v>
+        <v>400</v>
       </c>
       <c r="C11" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D11" s="4">
-        <v>0.03939814814814815</v>
+        <v>3.9398148148148147E-2</v>
       </c>
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
@@ -740,23 +749,23 @@
       <c r="M11" s="2"/>
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
-      <c r="P11" s="7"/>
-      <c r="Q11" s="7"/>
-      <c r="R11" s="7"/>
+      <c r="P11" s="2"/>
+      <c r="Q11" s="2"/>
+      <c r="R11" s="2"/>
       <c r="S11" s="2"/>
     </row>
-    <row r="12">
+    <row r="12" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B12" s="3">
-        <v>390.0</v>
+        <v>390</v>
       </c>
       <c r="C12" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D12" s="4">
-        <v>0.03756944444444445</v>
+        <v>3.7569444444444447E-2</v>
       </c>
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
@@ -769,23 +778,23 @@
       <c r="M12" s="2"/>
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
-      <c r="P12" s="7"/>
-      <c r="Q12" s="7"/>
-      <c r="R12" s="7"/>
+      <c r="P12" s="2"/>
+      <c r="Q12" s="2"/>
+      <c r="R12" s="2"/>
       <c r="S12" s="2"/>
     </row>
-    <row r="13">
+    <row r="13" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B13" s="3">
-        <v>380.0</v>
+        <v>380</v>
       </c>
       <c r="C13" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D13" s="4">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="E13" s="2"/>
       <c r="F13" s="2"/>
@@ -798,23 +807,23 @@
       <c r="M13" s="2"/>
       <c r="N13" s="2"/>
       <c r="O13" s="2"/>
-      <c r="P13" s="7"/>
-      <c r="Q13" s="7"/>
-      <c r="R13" s="7"/>
+      <c r="P13" s="2"/>
+      <c r="Q13" s="2"/>
+      <c r="R13" s="2"/>
       <c r="S13" s="2"/>
     </row>
-    <row r="14">
+    <row r="14" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B14" s="3">
-        <v>340.0</v>
+        <v>340</v>
       </c>
       <c r="C14" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D14" s="4">
-        <v>0.017997685185185186</v>
+        <v>1.7997685185185186E-2</v>
       </c>
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
@@ -827,23 +836,23 @@
       <c r="M14" s="2"/>
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
-      <c r="P14" s="7"/>
-      <c r="Q14" s="7"/>
-      <c r="R14" s="7"/>
+      <c r="P14" s="2"/>
+      <c r="Q14" s="2"/>
+      <c r="R14" s="2"/>
       <c r="S14" s="2"/>
     </row>
-    <row r="15">
+    <row r="15" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B15" s="3">
-        <v>300.0</v>
+        <v>300</v>
       </c>
       <c r="C15" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D15" s="4">
-        <v>0.04761574074074074</v>
+        <v>4.7615740740740743E-2</v>
       </c>
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
@@ -856,23 +865,23 @@
       <c r="M15" s="2"/>
       <c r="N15" s="2"/>
       <c r="O15" s="2"/>
-      <c r="P15" s="7"/>
-      <c r="Q15" s="7"/>
-      <c r="R15" s="7"/>
+      <c r="P15" s="2"/>
+      <c r="Q15" s="2"/>
+      <c r="R15" s="2"/>
       <c r="S15" s="2"/>
     </row>
-    <row r="16">
+    <row r="16" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B16" s="3">
-        <v>240.0</v>
+        <v>240</v>
       </c>
       <c r="C16" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D16" s="4">
-        <v>0.014641203703703703</v>
+        <v>1.4641203703703703E-2</v>
       </c>
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
@@ -885,23 +894,23 @@
       <c r="M16" s="2"/>
       <c r="N16" s="2"/>
       <c r="O16" s="2"/>
-      <c r="P16" s="7"/>
-      <c r="Q16" s="7"/>
-      <c r="R16" s="7"/>
+      <c r="P16" s="2"/>
+      <c r="Q16" s="2"/>
+      <c r="R16" s="2"/>
       <c r="S16" s="2"/>
     </row>
-    <row r="17">
+    <row r="17" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B17" s="3">
-        <v>240.0</v>
+        <v>240</v>
       </c>
       <c r="C17" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D17" s="4">
-        <v>0.044097222222222225</v>
+        <v>4.4097222222222225E-2</v>
       </c>
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
@@ -914,23 +923,23 @@
       <c r="M17" s="2"/>
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
-      <c r="P17" s="7"/>
-      <c r="Q17" s="7"/>
-      <c r="R17" s="7"/>
+      <c r="P17" s="2"/>
+      <c r="Q17" s="2"/>
+      <c r="R17" s="2"/>
       <c r="S17" s="2"/>
     </row>
-    <row r="18">
+    <row r="18" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B18" s="3">
-        <v>240.0</v>
+        <v>240</v>
       </c>
       <c r="C18" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D18" s="4">
-        <v>0.04832175925925926</v>
+        <v>4.8321759259259259E-2</v>
       </c>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
@@ -943,23 +952,23 @@
       <c r="M18" s="2"/>
       <c r="N18" s="2"/>
       <c r="O18" s="2"/>
-      <c r="P18" s="7"/>
-      <c r="Q18" s="7"/>
-      <c r="R18" s="7"/>
+      <c r="P18" s="2"/>
+      <c r="Q18" s="2"/>
+      <c r="R18" s="2"/>
       <c r="S18" s="2"/>
     </row>
-    <row r="19">
+    <row r="19" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B19" s="3">
-        <v>240.0</v>
+        <v>240</v>
       </c>
       <c r="C19" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D19" s="4">
-        <v>0.05855324074074074</v>
+        <v>5.8553240740740739E-2</v>
       </c>
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
@@ -972,23 +981,23 @@
       <c r="M19" s="2"/>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
-      <c r="P19" s="7"/>
-      <c r="Q19" s="7"/>
-      <c r="R19" s="7"/>
+      <c r="P19" s="2"/>
+      <c r="Q19" s="2"/>
+      <c r="R19" s="2"/>
       <c r="S19" s="2"/>
     </row>
-    <row r="20">
+    <row r="20" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B20" s="3">
-        <v>200.0</v>
+        <v>200</v>
       </c>
       <c r="C20" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D20" s="4">
-        <v>0.027395833333333335</v>
+        <v>2.7395833333333335E-2</v>
       </c>
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
@@ -1001,23 +1010,23 @@
       <c r="M20" s="2"/>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
-      <c r="P20" s="7"/>
-      <c r="Q20" s="7"/>
-      <c r="R20" s="7"/>
+      <c r="P20" s="2"/>
+      <c r="Q20" s="2"/>
+      <c r="R20" s="2"/>
       <c r="S20" s="2"/>
     </row>
-    <row r="21">
+    <row r="21" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B21" s="3">
-        <v>200.0</v>
+        <v>200</v>
       </c>
       <c r="C21" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D21" s="4">
-        <v>0.034375</v>
+        <v>3.4375000000000003E-2</v>
       </c>
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
@@ -1030,23 +1039,23 @@
       <c r="M21" s="2"/>
       <c r="N21" s="2"/>
       <c r="O21" s="2"/>
-      <c r="P21" s="7"/>
-      <c r="Q21" s="7"/>
-      <c r="R21" s="7"/>
+      <c r="P21" s="2"/>
+      <c r="Q21" s="2"/>
+      <c r="R21" s="2"/>
       <c r="S21" s="2"/>
     </row>
-    <row r="22">
+    <row r="22" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B22" s="3">
-        <v>200.0</v>
+        <v>200</v>
       </c>
       <c r="C22" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D22" s="4">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
@@ -1059,23 +1068,23 @@
       <c r="M22" s="2"/>
       <c r="N22" s="2"/>
       <c r="O22" s="2"/>
-      <c r="P22" s="7"/>
-      <c r="Q22" s="7"/>
-      <c r="R22" s="7"/>
+      <c r="P22" s="2"/>
+      <c r="Q22" s="2"/>
+      <c r="R22" s="2"/>
       <c r="S22" s="2"/>
     </row>
-    <row r="23">
+    <row r="23" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B23" s="3">
-        <v>190.0</v>
+        <v>190</v>
       </c>
       <c r="C23" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D23" s="4">
-        <v>0.014618055555555556</v>
+        <v>1.4618055555555556E-2</v>
       </c>
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
@@ -1088,23 +1097,23 @@
       <c r="M23" s="2"/>
       <c r="N23" s="2"/>
       <c r="O23" s="2"/>
-      <c r="P23" s="7"/>
-      <c r="Q23" s="7"/>
-      <c r="R23" s="7"/>
+      <c r="P23" s="2"/>
+      <c r="Q23" s="2"/>
+      <c r="R23" s="2"/>
       <c r="S23" s="2"/>
     </row>
-    <row r="24">
+    <row r="24" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B24" s="3">
-        <v>190.0</v>
+        <v>190</v>
       </c>
       <c r="C24" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D24" s="4">
-        <v>0.028819444444444446</v>
+        <v>2.8819444444444446E-2</v>
       </c>
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
@@ -1117,23 +1126,23 @@
       <c r="M24" s="2"/>
       <c r="N24" s="2"/>
       <c r="O24" s="2"/>
-      <c r="P24" s="7"/>
-      <c r="Q24" s="7"/>
-      <c r="R24" s="7"/>
+      <c r="P24" s="2"/>
+      <c r="Q24" s="2"/>
+      <c r="R24" s="2"/>
       <c r="S24" s="2"/>
     </row>
-    <row r="25">
+    <row r="25" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B25" s="3">
-        <v>150.0</v>
+        <v>150</v>
       </c>
       <c r="C25" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D25" s="4">
-        <v>0.03017361111111111</v>
+        <v>3.0173611111111109E-2</v>
       </c>
       <c r="E25" s="2"/>
       <c r="F25" s="2"/>
@@ -1146,23 +1155,23 @@
       <c r="M25" s="2"/>
       <c r="N25" s="2"/>
       <c r="O25" s="2"/>
-      <c r="P25" s="7"/>
-      <c r="Q25" s="7"/>
-      <c r="R25" s="7"/>
+      <c r="P25" s="2"/>
+      <c r="Q25" s="2"/>
+      <c r="R25" s="2"/>
       <c r="S25" s="2"/>
     </row>
-    <row r="26">
+    <row r="26" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B26" s="3">
-        <v>70.0</v>
+        <v>70</v>
       </c>
       <c r="C26" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D26" s="4">
-        <v>0.05116898148148148</v>
+        <v>5.1168981481481482E-2</v>
       </c>
       <c r="E26" s="2"/>
       <c r="F26" s="2"/>
@@ -1175,23 +1184,23 @@
       <c r="M26" s="2"/>
       <c r="N26" s="2"/>
       <c r="O26" s="2"/>
-      <c r="P26" s="7"/>
-      <c r="Q26" s="7"/>
-      <c r="R26" s="7"/>
+      <c r="P26" s="2"/>
+      <c r="Q26" s="2"/>
+      <c r="R26" s="2"/>
       <c r="S26" s="2"/>
     </row>
-    <row r="27">
+    <row r="27" spans="1:19" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B27" s="3">
-        <v>70.0</v>
+        <v>70</v>
       </c>
       <c r="C27" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D27" s="4">
-        <v>0.06251157407407408</v>
+        <v>6.2511574074074081E-2</v>
       </c>
       <c r="E27" s="2"/>
       <c r="F27" s="2"/>
@@ -1204,23 +1213,23 @@
       <c r="M27" s="2"/>
       <c r="N27" s="2"/>
       <c r="O27" s="2"/>
-      <c r="P27" s="7"/>
-      <c r="Q27" s="7"/>
-      <c r="R27" s="7"/>
+      <c r="P27" s="2"/>
+      <c r="Q27" s="2"/>
+      <c r="R27" s="2"/>
       <c r="S27" s="2"/>
     </row>
-    <row r="28">
+    <row r="28" spans="1:19" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B28" s="3">
-        <v>50.0</v>
+        <v>50</v>
       </c>
       <c r="C28" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D28" s="4">
-        <v>0.01673611111111111</v>
+        <v>1.6736111111111111E-2</v>
       </c>
       <c r="E28" s="2"/>
       <c r="F28" s="2"/>
@@ -1233,23 +1242,23 @@
       <c r="M28" s="2"/>
       <c r="N28" s="2"/>
       <c r="O28" s="2"/>
-      <c r="P28" s="7"/>
-      <c r="Q28" s="7"/>
-      <c r="R28" s="7"/>
+      <c r="P28" s="2"/>
+      <c r="Q28" s="2"/>
+      <c r="R28" s="2"/>
       <c r="S28" s="2"/>
     </row>
-    <row r="29">
+    <row r="29" spans="1:19" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B29" s="3">
-        <v>50.0</v>
+        <v>50</v>
       </c>
       <c r="C29" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D29" s="4">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="E29" s="2"/>
       <c r="F29" s="2"/>
@@ -1262,23 +1271,23 @@
       <c r="M29" s="2"/>
       <c r="N29" s="2"/>
       <c r="O29" s="2"/>
-      <c r="P29" s="7"/>
-      <c r="Q29" s="7"/>
-      <c r="R29" s="7"/>
+      <c r="P29" s="2"/>
+      <c r="Q29" s="2"/>
+      <c r="R29" s="2"/>
       <c r="S29" s="2"/>
     </row>
-    <row r="30">
+    <row r="30" spans="1:19" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B30" s="3">
-        <v>50.0</v>
+        <v>50</v>
       </c>
       <c r="C30" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D30" s="4">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="E30" s="2"/>
       <c r="F30" s="2"/>
@@ -1291,23 +1300,23 @@
       <c r="M30" s="2"/>
       <c r="N30" s="2"/>
       <c r="O30" s="2"/>
-      <c r="P30" s="7"/>
-      <c r="Q30" s="7"/>
-      <c r="R30" s="7"/>
+      <c r="P30" s="2"/>
+      <c r="Q30" s="2"/>
+      <c r="R30" s="2"/>
       <c r="S30" s="2"/>
     </row>
-    <row r="31">
+    <row r="31" spans="1:19" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B31" s="3">
-        <v>40.0</v>
+        <v>40</v>
       </c>
       <c r="C31" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D31" s="4">
-        <v>0.019965277777777776</v>
+        <v>1.9965277777777776E-2</v>
       </c>
       <c r="E31" s="2"/>
       <c r="F31" s="2"/>
@@ -1320,23 +1329,23 @@
       <c r="M31" s="2"/>
       <c r="N31" s="2"/>
       <c r="O31" s="2"/>
-      <c r="P31" s="7"/>
-      <c r="Q31" s="7"/>
-      <c r="R31" s="7"/>
+      <c r="P31" s="2"/>
+      <c r="Q31" s="2"/>
+      <c r="R31" s="2"/>
       <c r="S31" s="2"/>
     </row>
-    <row r="32">
+    <row r="32" spans="1:19" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B32" s="3">
-        <v>40.0</v>
+        <v>40</v>
       </c>
       <c r="C32" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D32" s="4">
-        <v>0.043993055555555556</v>
+        <v>4.3993055555555556E-2</v>
       </c>
       <c r="E32" s="2"/>
       <c r="F32" s="2"/>
@@ -1349,23 +1358,23 @@
       <c r="M32" s="2"/>
       <c r="N32" s="2"/>
       <c r="O32" s="2"/>
-      <c r="P32" s="7"/>
-      <c r="Q32" s="7"/>
-      <c r="R32" s="7"/>
+      <c r="P32" s="2"/>
+      <c r="Q32" s="2"/>
+      <c r="R32" s="2"/>
       <c r="S32" s="2"/>
     </row>
-    <row r="33">
+    <row r="33" spans="1:19" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B33" s="3">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C33" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D33" s="4">
-        <v>0.004398148148148148</v>
+        <v>4.3981481481481484E-3</v>
       </c>
       <c r="E33" s="2"/>
       <c r="F33" s="2"/>
@@ -1378,23 +1387,23 @@
       <c r="M33" s="2"/>
       <c r="N33" s="2"/>
       <c r="O33" s="2"/>
-      <c r="P33" s="7"/>
-      <c r="Q33" s="7"/>
-      <c r="R33" s="7"/>
+      <c r="P33" s="2"/>
+      <c r="Q33" s="2"/>
+      <c r="R33" s="2"/>
       <c r="S33" s="2"/>
     </row>
-    <row r="34">
+    <row r="34" spans="1:19" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B34" s="3">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C34" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D34" s="4">
-        <v>0.008541666666666666</v>
+        <v>8.5416666666666662E-3</v>
       </c>
       <c r="E34" s="2"/>
       <c r="F34" s="2"/>
@@ -1407,23 +1416,23 @@
       <c r="M34" s="2"/>
       <c r="N34" s="2"/>
       <c r="O34" s="2"/>
-      <c r="P34" s="7"/>
-      <c r="Q34" s="7"/>
-      <c r="R34" s="7"/>
+      <c r="P34" s="2"/>
+      <c r="Q34" s="2"/>
+      <c r="R34" s="2"/>
       <c r="S34" s="2"/>
     </row>
-    <row r="35">
+    <row r="35" spans="1:19" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B35" s="3">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C35" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D35" s="4">
-        <v>0.015104166666666667</v>
+        <v>1.5104166666666667E-2</v>
       </c>
       <c r="E35" s="2"/>
       <c r="F35" s="2"/>
@@ -1436,23 +1445,23 @@
       <c r="M35" s="2"/>
       <c r="N35" s="2"/>
       <c r="O35" s="2"/>
-      <c r="P35" s="7"/>
-      <c r="Q35" s="7"/>
-      <c r="R35" s="7"/>
+      <c r="P35" s="2"/>
+      <c r="Q35" s="2"/>
+      <c r="R35" s="2"/>
       <c r="S35" s="2"/>
     </row>
-    <row r="36">
+    <row r="36" spans="1:19" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B36" s="3">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C36" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D36" s="4">
-        <v>0.029907407407407407</v>
+        <v>2.9907407407407407E-2</v>
       </c>
       <c r="E36" s="2"/>
       <c r="F36" s="2"/>
@@ -1465,23 +1474,23 @@
       <c r="M36" s="2"/>
       <c r="N36" s="2"/>
       <c r="O36" s="2"/>
-      <c r="P36" s="7"/>
-      <c r="Q36" s="7"/>
-      <c r="R36" s="7"/>
+      <c r="P36" s="2"/>
+      <c r="Q36" s="2"/>
+      <c r="R36" s="2"/>
       <c r="S36" s="2"/>
     </row>
-    <row r="37">
+    <row r="37" spans="1:19" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B37" s="3">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C37" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D37" s="4">
-        <v>0.05219907407407407</v>
+        <v>5.2199074074074071E-2</v>
       </c>
       <c r="E37" s="2"/>
       <c r="F37" s="2"/>
@@ -1494,43 +1503,44 @@
       <c r="M37" s="2"/>
       <c r="N37" s="2"/>
       <c r="O37" s="2"/>
-      <c r="P37" s="7"/>
-      <c r="Q37" s="7"/>
-      <c r="R37" s="7"/>
+      <c r="P37" s="2"/>
+      <c r="Q37" s="2"/>
+      <c r="R37" s="2"/>
       <c r="S37" s="2"/>
     </row>
-    <row r="38">
+    <row r="38" spans="1:19" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B38" s="3">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="C38" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="D38" s="4">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="E38" s="2"/>
       <c r="F38" s="2"/>
       <c r="G38" s="2"/>
       <c r="H38" s="2"/>
-      <c r="I38" s="6"/>
+      <c r="I38" s="7"/>
+      <c r="J38" s="8"/>
       <c r="K38" s="3"/>
       <c r="L38" s="2"/>
       <c r="M38" s="2"/>
       <c r="N38" s="2"/>
       <c r="O38" s="2"/>
-      <c r="P38" s="7"/>
-      <c r="Q38" s="7"/>
-      <c r="R38" s="7"/>
+      <c r="P38" s="2"/>
+      <c r="Q38" s="2"/>
+      <c r="R38" s="2"/>
       <c r="S38" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="I38:J38"/>
   </mergeCells>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update: week 11 leaderboard
</commit_message>
<xml_diff>
--- a/frontend/public/weekly_contest_2_leaderboard_v2.xlsx
+++ b/frontend/public/weekly_contest_2_leaderboard_v2.xlsx
@@ -172,7 +172,7 @@
     <t xml:space="preserve">B. Shreya Kamath</t>
   </si>
   <si>
-    <t xml:space="preserve">bshreyakamath@gmail.com</t>
+    <t xml:space="preserve">nnm24am015@nmamit.in</t>
   </si>
   <si>
     <t xml:space="preserve">Shravya S</t>
@@ -308,16 +308,16 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="0"/>
     </font>
   </fonts>
   <fills count="2">
@@ -362,40 +362,44 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -591,46 +595,46 @@
   <dimension ref="A1:T38"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34.75"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16.75"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="16.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
-      <c r="P1" s="1"/>
-      <c r="Q1" s="1"/>
-      <c r="R1" s="1"/>
-      <c r="S1" s="1"/>
-      <c r="T1" s="1"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
+      <c r="O1" s="2"/>
+      <c r="P1" s="2"/>
+      <c r="Q1" s="2"/>
+      <c r="R1" s="2"/>
+      <c r="S1" s="2"/>
+      <c r="T1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -645,27 +649,27 @@
       <c r="E2" s="5" t="n">
         <v>0.0176388888888889</v>
       </c>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
       <c r="H2" s="6"/>
       <c r="I2" s="7"/>
       <c r="J2" s="7"/>
-      <c r="K2" s="2"/>
+      <c r="K2" s="3"/>
       <c r="L2" s="4"/>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2"/>
-      <c r="O2" s="2"/>
-      <c r="P2" s="2"/>
-      <c r="Q2" s="2"/>
-      <c r="R2" s="2"/>
-      <c r="S2" s="2"/>
-      <c r="T2" s="2"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="O2" s="3"/>
+      <c r="P2" s="3"/>
+      <c r="Q2" s="3"/>
+      <c r="R2" s="3"/>
+      <c r="S2" s="3"/>
+      <c r="T2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C3" s="4" t="n">
@@ -677,27 +681,27 @@
       <c r="E3" s="5" t="n">
         <v>0.0201736111111111</v>
       </c>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
       <c r="H3" s="6"/>
       <c r="I3" s="7"/>
       <c r="J3" s="7"/>
-      <c r="K3" s="2"/>
+      <c r="K3" s="3"/>
       <c r="L3" s="4"/>
-      <c r="M3" s="2"/>
-      <c r="N3" s="2"/>
-      <c r="O3" s="2"/>
-      <c r="P3" s="2"/>
-      <c r="Q3" s="2"/>
-      <c r="R3" s="2"/>
-      <c r="S3" s="2"/>
-      <c r="T3" s="2"/>
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
+      <c r="O3" s="3"/>
+      <c r="P3" s="3"/>
+      <c r="Q3" s="3"/>
+      <c r="R3" s="3"/>
+      <c r="S3" s="3"/>
+      <c r="T3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>10</v>
       </c>
       <c r="C4" s="4" t="n">
@@ -709,27 +713,27 @@
       <c r="E4" s="5" t="n">
         <v>0.0203009259259259</v>
       </c>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
       <c r="H4" s="6"/>
       <c r="I4" s="7"/>
       <c r="J4" s="7"/>
-      <c r="K4" s="2"/>
+      <c r="K4" s="3"/>
       <c r="L4" s="4"/>
-      <c r="M4" s="2"/>
-      <c r="N4" s="2"/>
-      <c r="O4" s="2"/>
-      <c r="P4" s="2"/>
-      <c r="Q4" s="2"/>
-      <c r="R4" s="2"/>
-      <c r="S4" s="2"/>
-      <c r="T4" s="2"/>
+      <c r="M4" s="3"/>
+      <c r="N4" s="3"/>
+      <c r="O4" s="3"/>
+      <c r="P4" s="3"/>
+      <c r="Q4" s="3"/>
+      <c r="R4" s="3"/>
+      <c r="S4" s="3"/>
+      <c r="T4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>12</v>
       </c>
       <c r="C5" s="4" t="n">
@@ -741,27 +745,27 @@
       <c r="E5" s="5" t="n">
         <v>0.0239236111111111</v>
       </c>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
       <c r="H5" s="6"/>
       <c r="I5" s="7"/>
       <c r="J5" s="7"/>
-      <c r="K5" s="2"/>
+      <c r="K5" s="3"/>
       <c r="L5" s="4"/>
-      <c r="M5" s="2"/>
-      <c r="N5" s="2"/>
-      <c r="O5" s="2"/>
-      <c r="P5" s="2"/>
-      <c r="Q5" s="2"/>
-      <c r="R5" s="2"/>
-      <c r="S5" s="2"/>
-      <c r="T5" s="2"/>
+      <c r="M5" s="3"/>
+      <c r="N5" s="3"/>
+      <c r="O5" s="3"/>
+      <c r="P5" s="3"/>
+      <c r="Q5" s="3"/>
+      <c r="R5" s="3"/>
+      <c r="S5" s="3"/>
+      <c r="T5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>14</v>
       </c>
       <c r="C6" s="4" t="n">
@@ -773,27 +777,27 @@
       <c r="E6" s="5" t="n">
         <v>0.0460763888888889</v>
       </c>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
       <c r="H6" s="6"/>
       <c r="I6" s="7"/>
       <c r="J6" s="7"/>
-      <c r="K6" s="2"/>
+      <c r="K6" s="3"/>
       <c r="L6" s="4"/>
-      <c r="M6" s="2"/>
-      <c r="N6" s="2"/>
-      <c r="O6" s="2"/>
-      <c r="P6" s="2"/>
-      <c r="Q6" s="2"/>
-      <c r="R6" s="2"/>
-      <c r="S6" s="2"/>
-      <c r="T6" s="2"/>
+      <c r="M6" s="3"/>
+      <c r="N6" s="3"/>
+      <c r="O6" s="3"/>
+      <c r="P6" s="3"/>
+      <c r="Q6" s="3"/>
+      <c r="R6" s="3"/>
+      <c r="S6" s="3"/>
+      <c r="T6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="3" t="s">
         <v>16</v>
       </c>
       <c r="C7" s="4" t="n">
@@ -805,27 +809,27 @@
       <c r="E7" s="5" t="n">
         <v>0.0315277777777778</v>
       </c>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
       <c r="H7" s="6"/>
       <c r="I7" s="7"/>
       <c r="J7" s="7"/>
-      <c r="K7" s="2"/>
+      <c r="K7" s="3"/>
       <c r="L7" s="4"/>
-      <c r="M7" s="2"/>
-      <c r="N7" s="2"/>
-      <c r="O7" s="2"/>
-      <c r="P7" s="2"/>
-      <c r="Q7" s="2"/>
-      <c r="R7" s="2"/>
-      <c r="S7" s="2"/>
-      <c r="T7" s="2"/>
+      <c r="M7" s="3"/>
+      <c r="N7" s="3"/>
+      <c r="O7" s="3"/>
+      <c r="P7" s="3"/>
+      <c r="Q7" s="3"/>
+      <c r="R7" s="3"/>
+      <c r="S7" s="3"/>
+      <c r="T7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="3" t="s">
         <v>18</v>
       </c>
       <c r="C8" s="4" t="n">
@@ -837,27 +841,27 @@
       <c r="E8" s="5" t="n">
         <v>0.0618402777777778</v>
       </c>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
       <c r="H8" s="6"/>
       <c r="I8" s="7"/>
       <c r="J8" s="7"/>
-      <c r="K8" s="2"/>
+      <c r="K8" s="3"/>
       <c r="L8" s="4"/>
-      <c r="M8" s="2"/>
-      <c r="N8" s="2"/>
-      <c r="O8" s="2"/>
-      <c r="P8" s="2"/>
-      <c r="Q8" s="2"/>
-      <c r="R8" s="2"/>
-      <c r="S8" s="2"/>
-      <c r="T8" s="2"/>
+      <c r="M8" s="3"/>
+      <c r="N8" s="3"/>
+      <c r="O8" s="3"/>
+      <c r="P8" s="3"/>
+      <c r="Q8" s="3"/>
+      <c r="R8" s="3"/>
+      <c r="S8" s="3"/>
+      <c r="T8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="3" t="s">
         <v>20</v>
       </c>
       <c r="C9" s="4" t="n">
@@ -869,27 +873,27 @@
       <c r="E9" s="5" t="n">
         <v>0.0443402777777778</v>
       </c>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
       <c r="H9" s="6"/>
       <c r="I9" s="7"/>
       <c r="J9" s="7"/>
-      <c r="K9" s="2"/>
+      <c r="K9" s="3"/>
       <c r="L9" s="4"/>
-      <c r="M9" s="2"/>
-      <c r="N9" s="2"/>
-      <c r="O9" s="2"/>
-      <c r="P9" s="2"/>
-      <c r="Q9" s="2"/>
-      <c r="R9" s="2"/>
-      <c r="S9" s="2"/>
-      <c r="T9" s="2"/>
+      <c r="M9" s="3"/>
+      <c r="N9" s="3"/>
+      <c r="O9" s="3"/>
+      <c r="P9" s="3"/>
+      <c r="Q9" s="3"/>
+      <c r="R9" s="3"/>
+      <c r="S9" s="3"/>
+      <c r="T9" s="3"/>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C10" s="4" t="n">
@@ -901,27 +905,27 @@
       <c r="E10" s="5" t="n">
         <v>0.0181018518518519</v>
       </c>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
       <c r="H10" s="6"/>
       <c r="I10" s="7"/>
       <c r="J10" s="7"/>
-      <c r="K10" s="2"/>
+      <c r="K10" s="3"/>
       <c r="L10" s="4"/>
-      <c r="M10" s="2"/>
-      <c r="N10" s="2"/>
-      <c r="O10" s="2"/>
-      <c r="P10" s="2"/>
-      <c r="Q10" s="2"/>
-      <c r="R10" s="2"/>
-      <c r="S10" s="2"/>
-      <c r="T10" s="2"/>
+      <c r="M10" s="3"/>
+      <c r="N10" s="3"/>
+      <c r="O10" s="3"/>
+      <c r="P10" s="3"/>
+      <c r="Q10" s="3"/>
+      <c r="R10" s="3"/>
+      <c r="S10" s="3"/>
+      <c r="T10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="3" t="s">
         <v>24</v>
       </c>
       <c r="C11" s="4" t="n">
@@ -933,27 +937,27 @@
       <c r="E11" s="5" t="n">
         <v>0.0393981481481482</v>
       </c>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
       <c r="H11" s="6"/>
       <c r="I11" s="7"/>
       <c r="J11" s="7"/>
-      <c r="K11" s="2"/>
+      <c r="K11" s="3"/>
       <c r="L11" s="4"/>
-      <c r="M11" s="2"/>
-      <c r="N11" s="2"/>
-      <c r="O11" s="2"/>
-      <c r="P11" s="2"/>
-      <c r="Q11" s="2"/>
-      <c r="R11" s="2"/>
-      <c r="S11" s="2"/>
-      <c r="T11" s="2"/>
+      <c r="M11" s="3"/>
+      <c r="N11" s="3"/>
+      <c r="O11" s="3"/>
+      <c r="P11" s="3"/>
+      <c r="Q11" s="3"/>
+      <c r="R11" s="3"/>
+      <c r="S11" s="3"/>
+      <c r="T11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="3" t="s">
         <v>26</v>
       </c>
       <c r="C12" s="4" t="n">
@@ -965,27 +969,27 @@
       <c r="E12" s="5" t="n">
         <v>0.0375694444444445</v>
       </c>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
       <c r="H12" s="6"/>
       <c r="I12" s="7"/>
       <c r="J12" s="7"/>
-      <c r="K12" s="2"/>
+      <c r="K12" s="3"/>
       <c r="L12" s="4"/>
-      <c r="M12" s="2"/>
-      <c r="N12" s="2"/>
-      <c r="O12" s="2"/>
-      <c r="P12" s="2"/>
-      <c r="Q12" s="2"/>
-      <c r="R12" s="2"/>
-      <c r="S12" s="2"/>
-      <c r="T12" s="2"/>
+      <c r="M12" s="3"/>
+      <c r="N12" s="3"/>
+      <c r="O12" s="3"/>
+      <c r="P12" s="3"/>
+      <c r="Q12" s="3"/>
+      <c r="R12" s="3"/>
+      <c r="S12" s="3"/>
+      <c r="T12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="3" t="s">
         <v>28</v>
       </c>
       <c r="C13" s="4" t="n">
@@ -997,27 +1001,27 @@
       <c r="E13" s="5" t="n">
         <v>0.0625</v>
       </c>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
       <c r="H13" s="6"/>
       <c r="I13" s="7"/>
       <c r="J13" s="7"/>
-      <c r="K13" s="2"/>
+      <c r="K13" s="3"/>
       <c r="L13" s="4"/>
-      <c r="M13" s="2"/>
-      <c r="N13" s="2"/>
-      <c r="O13" s="2"/>
-      <c r="P13" s="2"/>
-      <c r="Q13" s="2"/>
-      <c r="R13" s="2"/>
-      <c r="S13" s="2"/>
-      <c r="T13" s="2"/>
+      <c r="M13" s="3"/>
+      <c r="N13" s="3"/>
+      <c r="O13" s="3"/>
+      <c r="P13" s="3"/>
+      <c r="Q13" s="3"/>
+      <c r="R13" s="3"/>
+      <c r="S13" s="3"/>
+      <c r="T13" s="3"/>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="3" t="s">
         <v>30</v>
       </c>
       <c r="C14" s="4" t="n">
@@ -1029,27 +1033,27 @@
       <c r="E14" s="5" t="n">
         <v>0.0179976851851852</v>
       </c>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
       <c r="H14" s="6"/>
       <c r="I14" s="7"/>
       <c r="J14" s="7"/>
-      <c r="K14" s="2"/>
+      <c r="K14" s="3"/>
       <c r="L14" s="4"/>
-      <c r="M14" s="2"/>
-      <c r="N14" s="2"/>
-      <c r="O14" s="2"/>
-      <c r="P14" s="2"/>
-      <c r="Q14" s="2"/>
-      <c r="R14" s="2"/>
-      <c r="S14" s="2"/>
-      <c r="T14" s="2"/>
+      <c r="M14" s="3"/>
+      <c r="N14" s="3"/>
+      <c r="O14" s="3"/>
+      <c r="P14" s="3"/>
+      <c r="Q14" s="3"/>
+      <c r="R14" s="3"/>
+      <c r="S14" s="3"/>
+      <c r="T14" s="3"/>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="3" t="s">
         <v>32</v>
       </c>
       <c r="C15" s="4" t="n">
@@ -1061,27 +1065,27 @@
       <c r="E15" s="5" t="n">
         <v>0.0476157407407407</v>
       </c>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
       <c r="H15" s="6"/>
       <c r="I15" s="7"/>
       <c r="J15" s="7"/>
-      <c r="K15" s="2"/>
+      <c r="K15" s="3"/>
       <c r="L15" s="4"/>
-      <c r="M15" s="2"/>
-      <c r="N15" s="2"/>
-      <c r="O15" s="2"/>
-      <c r="P15" s="2"/>
-      <c r="Q15" s="2"/>
-      <c r="R15" s="2"/>
-      <c r="S15" s="2"/>
-      <c r="T15" s="2"/>
+      <c r="M15" s="3"/>
+      <c r="N15" s="3"/>
+      <c r="O15" s="3"/>
+      <c r="P15" s="3"/>
+      <c r="Q15" s="3"/>
+      <c r="R15" s="3"/>
+      <c r="S15" s="3"/>
+      <c r="T15" s="3"/>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="3" t="s">
         <v>34</v>
       </c>
       <c r="C16" s="4" t="n">
@@ -1093,27 +1097,27 @@
       <c r="E16" s="5" t="n">
         <v>0.0146412037037037</v>
       </c>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
       <c r="H16" s="6"/>
       <c r="I16" s="7"/>
       <c r="J16" s="7"/>
-      <c r="K16" s="2"/>
+      <c r="K16" s="3"/>
       <c r="L16" s="4"/>
-      <c r="M16" s="2"/>
-      <c r="N16" s="2"/>
-      <c r="O16" s="2"/>
-      <c r="P16" s="2"/>
-      <c r="Q16" s="2"/>
-      <c r="R16" s="2"/>
-      <c r="S16" s="2"/>
-      <c r="T16" s="2"/>
+      <c r="M16" s="3"/>
+      <c r="N16" s="3"/>
+      <c r="O16" s="3"/>
+      <c r="P16" s="3"/>
+      <c r="Q16" s="3"/>
+      <c r="R16" s="3"/>
+      <c r="S16" s="3"/>
+      <c r="T16" s="3"/>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="3" t="s">
         <v>36</v>
       </c>
       <c r="C17" s="4" t="n">
@@ -1125,27 +1129,27 @@
       <c r="E17" s="5" t="n">
         <v>0.0440972222222222</v>
       </c>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
       <c r="H17" s="6"/>
       <c r="I17" s="7"/>
       <c r="J17" s="7"/>
-      <c r="K17" s="2"/>
+      <c r="K17" s="3"/>
       <c r="L17" s="4"/>
-      <c r="M17" s="2"/>
-      <c r="N17" s="2"/>
-      <c r="O17" s="2"/>
-      <c r="P17" s="2"/>
-      <c r="Q17" s="2"/>
-      <c r="R17" s="2"/>
-      <c r="S17" s="2"/>
-      <c r="T17" s="2"/>
+      <c r="M17" s="3"/>
+      <c r="N17" s="3"/>
+      <c r="O17" s="3"/>
+      <c r="P17" s="3"/>
+      <c r="Q17" s="3"/>
+      <c r="R17" s="3"/>
+      <c r="S17" s="3"/>
+      <c r="T17" s="3"/>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="3" t="s">
         <v>38</v>
       </c>
       <c r="C18" s="4" t="n">
@@ -1157,27 +1161,27 @@
       <c r="E18" s="5" t="n">
         <v>0.0483217592592593</v>
       </c>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
       <c r="H18" s="6"/>
       <c r="I18" s="7"/>
       <c r="J18" s="7"/>
-      <c r="K18" s="2"/>
+      <c r="K18" s="3"/>
       <c r="L18" s="4"/>
-      <c r="M18" s="2"/>
-      <c r="N18" s="2"/>
-      <c r="O18" s="2"/>
-      <c r="P18" s="2"/>
-      <c r="Q18" s="2"/>
-      <c r="R18" s="2"/>
-      <c r="S18" s="2"/>
-      <c r="T18" s="2"/>
+      <c r="M18" s="3"/>
+      <c r="N18" s="3"/>
+      <c r="O18" s="3"/>
+      <c r="P18" s="3"/>
+      <c r="Q18" s="3"/>
+      <c r="R18" s="3"/>
+      <c r="S18" s="3"/>
+      <c r="T18" s="3"/>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="3" t="s">
         <v>40</v>
       </c>
       <c r="C19" s="4" t="n">
@@ -1189,27 +1193,27 @@
       <c r="E19" s="5" t="n">
         <v>0.0585532407407407</v>
       </c>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
       <c r="H19" s="6"/>
       <c r="I19" s="7"/>
       <c r="J19" s="7"/>
-      <c r="K19" s="2"/>
+      <c r="K19" s="3"/>
       <c r="L19" s="4"/>
-      <c r="M19" s="2"/>
-      <c r="N19" s="2"/>
-      <c r="O19" s="2"/>
-      <c r="P19" s="2"/>
-      <c r="Q19" s="2"/>
-      <c r="R19" s="2"/>
-      <c r="S19" s="2"/>
-      <c r="T19" s="2"/>
+      <c r="M19" s="3"/>
+      <c r="N19" s="3"/>
+      <c r="O19" s="3"/>
+      <c r="P19" s="3"/>
+      <c r="Q19" s="3"/>
+      <c r="R19" s="3"/>
+      <c r="S19" s="3"/>
+      <c r="T19" s="3"/>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2" t="s">
+      <c r="A20" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="3" t="s">
         <v>42</v>
       </c>
       <c r="C20" s="4" t="n">
@@ -1221,27 +1225,27 @@
       <c r="E20" s="5" t="n">
         <v>0.0273958333333333</v>
       </c>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
       <c r="H20" s="6"/>
       <c r="I20" s="7"/>
       <c r="J20" s="7"/>
-      <c r="K20" s="2"/>
+      <c r="K20" s="3"/>
       <c r="L20" s="4"/>
-      <c r="M20" s="2"/>
-      <c r="N20" s="2"/>
-      <c r="O20" s="2"/>
-      <c r="P20" s="2"/>
-      <c r="Q20" s="2"/>
-      <c r="R20" s="2"/>
-      <c r="S20" s="2"/>
-      <c r="T20" s="2"/>
+      <c r="M20" s="3"/>
+      <c r="N20" s="3"/>
+      <c r="O20" s="3"/>
+      <c r="P20" s="3"/>
+      <c r="Q20" s="3"/>
+      <c r="R20" s="3"/>
+      <c r="S20" s="3"/>
+      <c r="T20" s="3"/>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2" t="s">
+      <c r="A21" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="3" t="s">
         <v>44</v>
       </c>
       <c r="C21" s="4" t="n">
@@ -1253,27 +1257,27 @@
       <c r="E21" s="5" t="n">
         <v>0.034375</v>
       </c>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
       <c r="H21" s="6"/>
       <c r="I21" s="7"/>
       <c r="J21" s="7"/>
-      <c r="K21" s="2"/>
+      <c r="K21" s="3"/>
       <c r="L21" s="4"/>
-      <c r="M21" s="2"/>
-      <c r="N21" s="2"/>
-      <c r="O21" s="2"/>
-      <c r="P21" s="2"/>
-      <c r="Q21" s="2"/>
-      <c r="R21" s="2"/>
-      <c r="S21" s="2"/>
-      <c r="T21" s="2"/>
+      <c r="M21" s="3"/>
+      <c r="N21" s="3"/>
+      <c r="O21" s="3"/>
+      <c r="P21" s="3"/>
+      <c r="Q21" s="3"/>
+      <c r="R21" s="3"/>
+      <c r="S21" s="3"/>
+      <c r="T21" s="3"/>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2" t="s">
+      <c r="A22" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="3" t="s">
         <v>46</v>
       </c>
       <c r="C22" s="4" t="n">
@@ -1285,27 +1289,27 @@
       <c r="E22" s="5" t="n">
         <v>0.0625</v>
       </c>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
       <c r="H22" s="6"/>
       <c r="I22" s="7"/>
       <c r="J22" s="7"/>
-      <c r="K22" s="2"/>
+      <c r="K22" s="3"/>
       <c r="L22" s="4"/>
-      <c r="M22" s="2"/>
-      <c r="N22" s="2"/>
-      <c r="O22" s="2"/>
-      <c r="P22" s="2"/>
-      <c r="Q22" s="2"/>
-      <c r="R22" s="2"/>
-      <c r="S22" s="2"/>
-      <c r="T22" s="2"/>
+      <c r="M22" s="3"/>
+      <c r="N22" s="3"/>
+      <c r="O22" s="3"/>
+      <c r="P22" s="3"/>
+      <c r="Q22" s="3"/>
+      <c r="R22" s="3"/>
+      <c r="S22" s="3"/>
+      <c r="T22" s="3"/>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
+      <c r="A23" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B23" s="3" t="s">
         <v>48</v>
       </c>
       <c r="C23" s="4" t="n">
@@ -1317,27 +1321,27 @@
       <c r="E23" s="5" t="n">
         <v>0.0146180555555556</v>
       </c>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
       <c r="H23" s="6"/>
       <c r="I23" s="7"/>
       <c r="J23" s="7"/>
-      <c r="K23" s="2"/>
+      <c r="K23" s="3"/>
       <c r="L23" s="4"/>
-      <c r="M23" s="2"/>
-      <c r="N23" s="2"/>
-      <c r="O23" s="2"/>
-      <c r="P23" s="2"/>
-      <c r="Q23" s="2"/>
-      <c r="R23" s="2"/>
-      <c r="S23" s="2"/>
-      <c r="T23" s="2"/>
+      <c r="M23" s="3"/>
+      <c r="N23" s="3"/>
+      <c r="O23" s="3"/>
+      <c r="P23" s="3"/>
+      <c r="Q23" s="3"/>
+      <c r="R23" s="3"/>
+      <c r="S23" s="3"/>
+      <c r="T23" s="3"/>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2" t="s">
+      <c r="A24" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="8" t="s">
         <v>50</v>
       </c>
       <c r="C24" s="4" t="n">
@@ -1349,27 +1353,27 @@
       <c r="E24" s="5" t="n">
         <v>0.0288194444444444</v>
       </c>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
       <c r="H24" s="6"/>
       <c r="I24" s="7"/>
       <c r="J24" s="7"/>
-      <c r="K24" s="2"/>
+      <c r="K24" s="3"/>
       <c r="L24" s="4"/>
-      <c r="M24" s="2"/>
-      <c r="N24" s="2"/>
-      <c r="O24" s="2"/>
-      <c r="P24" s="2"/>
-      <c r="Q24" s="2"/>
-      <c r="R24" s="2"/>
-      <c r="S24" s="2"/>
-      <c r="T24" s="2"/>
+      <c r="M24" s="3"/>
+      <c r="N24" s="3"/>
+      <c r="O24" s="3"/>
+      <c r="P24" s="3"/>
+      <c r="Q24" s="3"/>
+      <c r="R24" s="3"/>
+      <c r="S24" s="3"/>
+      <c r="T24" s="3"/>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2" t="s">
+      <c r="A25" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B25" s="3" t="s">
         <v>52</v>
       </c>
       <c r="C25" s="4" t="n">
@@ -1381,27 +1385,27 @@
       <c r="E25" s="5" t="n">
         <v>0.0301736111111111</v>
       </c>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
       <c r="H25" s="6"/>
       <c r="I25" s="7"/>
       <c r="J25" s="7"/>
-      <c r="K25" s="2"/>
+      <c r="K25" s="3"/>
       <c r="L25" s="4"/>
-      <c r="M25" s="2"/>
-      <c r="N25" s="2"/>
-      <c r="O25" s="2"/>
-      <c r="P25" s="2"/>
-      <c r="Q25" s="2"/>
-      <c r="R25" s="2"/>
-      <c r="S25" s="2"/>
-      <c r="T25" s="2"/>
+      <c r="M25" s="3"/>
+      <c r="N25" s="3"/>
+      <c r="O25" s="3"/>
+      <c r="P25" s="3"/>
+      <c r="Q25" s="3"/>
+      <c r="R25" s="3"/>
+      <c r="S25" s="3"/>
+      <c r="T25" s="3"/>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2" t="s">
+      <c r="A26" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="3" t="s">
         <v>54</v>
       </c>
       <c r="C26" s="4" t="n">
@@ -1413,27 +1417,27 @@
       <c r="E26" s="5" t="n">
         <v>0.0511689814814815</v>
       </c>
-      <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
       <c r="H26" s="6"/>
       <c r="I26" s="7"/>
       <c r="J26" s="7"/>
-      <c r="K26" s="2"/>
+      <c r="K26" s="3"/>
       <c r="L26" s="4"/>
-      <c r="M26" s="2"/>
-      <c r="N26" s="2"/>
-      <c r="O26" s="2"/>
-      <c r="P26" s="2"/>
-      <c r="Q26" s="2"/>
-      <c r="R26" s="2"/>
-      <c r="S26" s="2"/>
-      <c r="T26" s="2"/>
+      <c r="M26" s="3"/>
+      <c r="N26" s="3"/>
+      <c r="O26" s="3"/>
+      <c r="P26" s="3"/>
+      <c r="Q26" s="3"/>
+      <c r="R26" s="3"/>
+      <c r="S26" s="3"/>
+      <c r="T26" s="3"/>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="2" t="s">
+      <c r="A27" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B27" s="3" t="s">
         <v>56</v>
       </c>
       <c r="C27" s="4" t="n">
@@ -1445,27 +1449,27 @@
       <c r="E27" s="5" t="n">
         <v>0.0625115740740741</v>
       </c>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
       <c r="H27" s="6"/>
       <c r="I27" s="7"/>
       <c r="J27" s="7"/>
-      <c r="K27" s="2"/>
+      <c r="K27" s="3"/>
       <c r="L27" s="4"/>
-      <c r="M27" s="2"/>
-      <c r="N27" s="2"/>
-      <c r="O27" s="2"/>
-      <c r="P27" s="2"/>
-      <c r="Q27" s="2"/>
-      <c r="R27" s="2"/>
-      <c r="S27" s="2"/>
-      <c r="T27" s="2"/>
+      <c r="M27" s="3"/>
+      <c r="N27" s="3"/>
+      <c r="O27" s="3"/>
+      <c r="P27" s="3"/>
+      <c r="Q27" s="3"/>
+      <c r="R27" s="3"/>
+      <c r="S27" s="3"/>
+      <c r="T27" s="3"/>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2" t="s">
+      <c r="A28" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B28" s="3" t="s">
         <v>58</v>
       </c>
       <c r="C28" s="4" t="n">
@@ -1477,27 +1481,27 @@
       <c r="E28" s="5" t="n">
         <v>0.0167361111111111</v>
       </c>
-      <c r="F28" s="2"/>
-      <c r="G28" s="2"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
       <c r="H28" s="6"/>
       <c r="I28" s="7"/>
       <c r="J28" s="7"/>
-      <c r="K28" s="2"/>
+      <c r="K28" s="3"/>
       <c r="L28" s="4"/>
-      <c r="M28" s="2"/>
-      <c r="N28" s="2"/>
-      <c r="O28" s="2"/>
-      <c r="P28" s="2"/>
-      <c r="Q28" s="2"/>
-      <c r="R28" s="2"/>
-      <c r="S28" s="2"/>
-      <c r="T28" s="2"/>
+      <c r="M28" s="3"/>
+      <c r="N28" s="3"/>
+      <c r="O28" s="3"/>
+      <c r="P28" s="3"/>
+      <c r="Q28" s="3"/>
+      <c r="R28" s="3"/>
+      <c r="S28" s="3"/>
+      <c r="T28" s="3"/>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="2" t="s">
+      <c r="A29" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="B29" s="3" t="s">
         <v>60</v>
       </c>
       <c r="C29" s="4" t="n">
@@ -1509,27 +1513,27 @@
       <c r="E29" s="5" t="n">
         <v>0.0625</v>
       </c>
-      <c r="F29" s="2"/>
-      <c r="G29" s="2"/>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3"/>
       <c r="H29" s="6"/>
       <c r="I29" s="7"/>
       <c r="J29" s="7"/>
-      <c r="K29" s="2"/>
+      <c r="K29" s="3"/>
       <c r="L29" s="4"/>
-      <c r="M29" s="2"/>
-      <c r="N29" s="2"/>
-      <c r="O29" s="2"/>
-      <c r="P29" s="2"/>
-      <c r="Q29" s="2"/>
-      <c r="R29" s="2"/>
-      <c r="S29" s="2"/>
-      <c r="T29" s="2"/>
+      <c r="M29" s="3"/>
+      <c r="N29" s="3"/>
+      <c r="O29" s="3"/>
+      <c r="P29" s="3"/>
+      <c r="Q29" s="3"/>
+      <c r="R29" s="3"/>
+      <c r="S29" s="3"/>
+      <c r="T29" s="3"/>
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="2" t="s">
+      <c r="A30" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="B30" s="3" t="s">
         <v>62</v>
       </c>
       <c r="C30" s="4" t="n">
@@ -1541,27 +1545,27 @@
       <c r="E30" s="5" t="n">
         <v>0.0625</v>
       </c>
-      <c r="F30" s="2"/>
-      <c r="G30" s="2"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
       <c r="H30" s="6"/>
       <c r="I30" s="7"/>
       <c r="J30" s="7"/>
-      <c r="K30" s="2"/>
+      <c r="K30" s="3"/>
       <c r="L30" s="4"/>
-      <c r="M30" s="2"/>
-      <c r="N30" s="2"/>
-      <c r="O30" s="2"/>
-      <c r="P30" s="2"/>
-      <c r="Q30" s="2"/>
-      <c r="R30" s="2"/>
-      <c r="S30" s="2"/>
-      <c r="T30" s="2"/>
+      <c r="M30" s="3"/>
+      <c r="N30" s="3"/>
+      <c r="O30" s="3"/>
+      <c r="P30" s="3"/>
+      <c r="Q30" s="3"/>
+      <c r="R30" s="3"/>
+      <c r="S30" s="3"/>
+      <c r="T30" s="3"/>
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="2" t="s">
+      <c r="A31" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="B31" s="3" t="s">
         <v>64</v>
       </c>
       <c r="C31" s="4" t="n">
@@ -1573,27 +1577,27 @@
       <c r="E31" s="5" t="n">
         <v>0.0199652777777778</v>
       </c>
-      <c r="F31" s="2"/>
-      <c r="G31" s="2"/>
+      <c r="F31" s="3"/>
+      <c r="G31" s="3"/>
       <c r="H31" s="6"/>
       <c r="I31" s="7"/>
       <c r="J31" s="7"/>
-      <c r="K31" s="2"/>
+      <c r="K31" s="3"/>
       <c r="L31" s="4"/>
-      <c r="M31" s="2"/>
-      <c r="N31" s="2"/>
-      <c r="O31" s="2"/>
-      <c r="P31" s="2"/>
-      <c r="Q31" s="2"/>
-      <c r="R31" s="2"/>
-      <c r="S31" s="2"/>
-      <c r="T31" s="2"/>
+      <c r="M31" s="3"/>
+      <c r="N31" s="3"/>
+      <c r="O31" s="3"/>
+      <c r="P31" s="3"/>
+      <c r="Q31" s="3"/>
+      <c r="R31" s="3"/>
+      <c r="S31" s="3"/>
+      <c r="T31" s="3"/>
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="2" t="s">
+      <c r="A32" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B32" s="3" t="s">
         <v>66</v>
       </c>
       <c r="C32" s="4" t="n">
@@ -1605,27 +1609,27 @@
       <c r="E32" s="5" t="n">
         <v>0.0439930555555556</v>
       </c>
-      <c r="F32" s="2"/>
-      <c r="G32" s="2"/>
+      <c r="F32" s="3"/>
+      <c r="G32" s="3"/>
       <c r="H32" s="6"/>
       <c r="I32" s="7"/>
       <c r="J32" s="7"/>
-      <c r="K32" s="2"/>
+      <c r="K32" s="3"/>
       <c r="L32" s="4"/>
-      <c r="M32" s="2"/>
-      <c r="N32" s="2"/>
-      <c r="O32" s="2"/>
-      <c r="P32" s="2"/>
-      <c r="Q32" s="2"/>
-      <c r="R32" s="2"/>
-      <c r="S32" s="2"/>
-      <c r="T32" s="2"/>
+      <c r="M32" s="3"/>
+      <c r="N32" s="3"/>
+      <c r="O32" s="3"/>
+      <c r="P32" s="3"/>
+      <c r="Q32" s="3"/>
+      <c r="R32" s="3"/>
+      <c r="S32" s="3"/>
+      <c r="T32" s="3"/>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="2" t="s">
+      <c r="A33" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="B33" s="3" t="s">
         <v>68</v>
       </c>
       <c r="C33" s="4" t="n">
@@ -1637,27 +1641,27 @@
       <c r="E33" s="5" t="n">
         <v>0.00439814814814815</v>
       </c>
-      <c r="F33" s="2"/>
-      <c r="G33" s="2"/>
-      <c r="H33" s="2"/>
-      <c r="I33" s="2"/>
+      <c r="F33" s="3"/>
+      <c r="G33" s="3"/>
+      <c r="H33" s="3"/>
+      <c r="I33" s="3"/>
       <c r="J33" s="7"/>
-      <c r="K33" s="2"/>
+      <c r="K33" s="3"/>
       <c r="L33" s="4"/>
-      <c r="M33" s="2"/>
-      <c r="N33" s="2"/>
-      <c r="O33" s="2"/>
-      <c r="P33" s="2"/>
-      <c r="Q33" s="2"/>
-      <c r="R33" s="2"/>
-      <c r="S33" s="2"/>
-      <c r="T33" s="2"/>
+      <c r="M33" s="3"/>
+      <c r="N33" s="3"/>
+      <c r="O33" s="3"/>
+      <c r="P33" s="3"/>
+      <c r="Q33" s="3"/>
+      <c r="R33" s="3"/>
+      <c r="S33" s="3"/>
+      <c r="T33" s="3"/>
     </row>
     <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="2" t="s">
+      <c r="A34" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="B34" s="3" t="s">
         <v>70</v>
       </c>
       <c r="C34" s="4" t="n">
@@ -1669,27 +1673,27 @@
       <c r="E34" s="5" t="n">
         <v>0.00854166666666667</v>
       </c>
-      <c r="F34" s="2"/>
-      <c r="G34" s="2"/>
-      <c r="H34" s="2"/>
-      <c r="I34" s="2"/>
+      <c r="F34" s="3"/>
+      <c r="G34" s="3"/>
+      <c r="H34" s="3"/>
+      <c r="I34" s="3"/>
       <c r="J34" s="7"/>
-      <c r="K34" s="2"/>
+      <c r="K34" s="3"/>
       <c r="L34" s="4"/>
-      <c r="M34" s="2"/>
-      <c r="N34" s="2"/>
-      <c r="O34" s="2"/>
-      <c r="P34" s="2"/>
-      <c r="Q34" s="2"/>
-      <c r="R34" s="2"/>
-      <c r="S34" s="2"/>
-      <c r="T34" s="2"/>
+      <c r="M34" s="3"/>
+      <c r="N34" s="3"/>
+      <c r="O34" s="3"/>
+      <c r="P34" s="3"/>
+      <c r="Q34" s="3"/>
+      <c r="R34" s="3"/>
+      <c r="S34" s="3"/>
+      <c r="T34" s="3"/>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="2" t="s">
+      <c r="A35" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="B35" s="3" t="s">
         <v>72</v>
       </c>
       <c r="C35" s="4" t="n">
@@ -1701,27 +1705,27 @@
       <c r="E35" s="5" t="n">
         <v>0.0151041666666667</v>
       </c>
-      <c r="F35" s="2"/>
-      <c r="G35" s="2"/>
-      <c r="H35" s="2"/>
-      <c r="I35" s="2"/>
+      <c r="F35" s="3"/>
+      <c r="G35" s="3"/>
+      <c r="H35" s="3"/>
+      <c r="I35" s="3"/>
       <c r="J35" s="7"/>
-      <c r="K35" s="2"/>
+      <c r="K35" s="3"/>
       <c r="L35" s="4"/>
-      <c r="M35" s="2"/>
-      <c r="N35" s="2"/>
-      <c r="O35" s="2"/>
-      <c r="P35" s="2"/>
-      <c r="Q35" s="2"/>
-      <c r="R35" s="2"/>
-      <c r="S35" s="2"/>
-      <c r="T35" s="2"/>
+      <c r="M35" s="3"/>
+      <c r="N35" s="3"/>
+      <c r="O35" s="3"/>
+      <c r="P35" s="3"/>
+      <c r="Q35" s="3"/>
+      <c r="R35" s="3"/>
+      <c r="S35" s="3"/>
+      <c r="T35" s="3"/>
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="2" t="s">
+      <c r="A36" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="B36" s="3" t="s">
         <v>74</v>
       </c>
       <c r="C36" s="4" t="n">
@@ -1733,27 +1737,27 @@
       <c r="E36" s="5" t="n">
         <v>0.0299074074074074</v>
       </c>
-      <c r="F36" s="2"/>
-      <c r="G36" s="2"/>
-      <c r="H36" s="2"/>
-      <c r="I36" s="2"/>
+      <c r="F36" s="3"/>
+      <c r="G36" s="3"/>
+      <c r="H36" s="3"/>
+      <c r="I36" s="3"/>
       <c r="J36" s="7"/>
-      <c r="K36" s="2"/>
+      <c r="K36" s="3"/>
       <c r="L36" s="4"/>
-      <c r="M36" s="2"/>
-      <c r="N36" s="2"/>
-      <c r="O36" s="2"/>
-      <c r="P36" s="2"/>
-      <c r="Q36" s="2"/>
-      <c r="R36" s="2"/>
-      <c r="S36" s="2"/>
-      <c r="T36" s="2"/>
+      <c r="M36" s="3"/>
+      <c r="N36" s="3"/>
+      <c r="O36" s="3"/>
+      <c r="P36" s="3"/>
+      <c r="Q36" s="3"/>
+      <c r="R36" s="3"/>
+      <c r="S36" s="3"/>
+      <c r="T36" s="3"/>
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="2" t="s">
+      <c r="A37" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="B37" s="2" t="s">
+      <c r="B37" s="3" t="s">
         <v>76</v>
       </c>
       <c r="C37" s="4" t="n">
@@ -1765,27 +1769,27 @@
       <c r="E37" s="5" t="n">
         <v>0.0521990740740741</v>
       </c>
-      <c r="F37" s="2"/>
-      <c r="G37" s="2"/>
-      <c r="H37" s="2"/>
-      <c r="I37" s="2"/>
+      <c r="F37" s="3"/>
+      <c r="G37" s="3"/>
+      <c r="H37" s="3"/>
+      <c r="I37" s="3"/>
       <c r="J37" s="7"/>
-      <c r="K37" s="2"/>
+      <c r="K37" s="3"/>
       <c r="L37" s="4"/>
-      <c r="M37" s="2"/>
-      <c r="N37" s="2"/>
-      <c r="O37" s="2"/>
-      <c r="P37" s="2"/>
-      <c r="Q37" s="2"/>
-      <c r="R37" s="2"/>
-      <c r="S37" s="2"/>
-      <c r="T37" s="2"/>
+      <c r="M37" s="3"/>
+      <c r="N37" s="3"/>
+      <c r="O37" s="3"/>
+      <c r="P37" s="3"/>
+      <c r="Q37" s="3"/>
+      <c r="R37" s="3"/>
+      <c r="S37" s="3"/>
+      <c r="T37" s="3"/>
     </row>
     <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="2" t="s">
+      <c r="A38" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="B38" s="3" t="s">
         <v>78</v>
       </c>
       <c r="C38" s="4" t="n">
@@ -1797,21 +1801,21 @@
       <c r="E38" s="5" t="n">
         <v>0.0625</v>
       </c>
-      <c r="F38" s="2"/>
-      <c r="G38" s="2"/>
-      <c r="H38" s="2"/>
-      <c r="I38" s="2"/>
-      <c r="J38" s="8"/>
-      <c r="K38" s="8"/>
+      <c r="F38" s="3"/>
+      <c r="G38" s="3"/>
+      <c r="H38" s="3"/>
+      <c r="I38" s="3"/>
+      <c r="J38" s="9"/>
+      <c r="K38" s="9"/>
       <c r="L38" s="4"/>
-      <c r="M38" s="2"/>
-      <c r="N38" s="2"/>
-      <c r="O38" s="2"/>
-      <c r="P38" s="2"/>
-      <c r="Q38" s="2"/>
-      <c r="R38" s="2"/>
-      <c r="S38" s="2"/>
-      <c r="T38" s="2"/>
+      <c r="M38" s="3"/>
+      <c r="N38" s="3"/>
+      <c r="O38" s="3"/>
+      <c r="P38" s="3"/>
+      <c r="Q38" s="3"/>
+      <c r="R38" s="3"/>
+      <c r="S38" s="3"/>
+      <c r="T38" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1819,6 +1823,7 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" display="sandeeppaikulyadi05@gmail.com"/>
+    <hyperlink ref="B24" r:id="rId2" display="nnm24am015@nmamit.in"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>